<commit_message>
feat: introduce initial LOS automation project including add-on supplement processing, core utilities, and GUI components.
</commit_message>
<xml_diff>
--- a/Data/LOSData.xlsx
+++ b/Data/LOSData.xlsx
@@ -1029,17 +1029,17 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>MANA RIDHA</t>
+          <t>Brianna Joe</t>
         </is>
       </c>
       <c r="H2" s="20" t="inlineStr">
         <is>
-          <t>FINN</t>
+          <t>Brianna Joe</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>FINN</t>
+          <t>Brianna</t>
         </is>
       </c>
       <c r="J2" s="22" t="n">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="P2" s="28" t="inlineStr">
         <is>
-          <t>8471291161908710</t>
+          <t>4428444224168525</t>
         </is>
       </c>
       <c r="Q2" s="25" t="n">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="T2" s="20" t="inlineStr">
         <is>
-          <t>James Morgan</t>
+          <t>Levi Ward</t>
         </is>
       </c>
       <c r="U2" s="25" t="n">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="AK2" s="28" t="inlineStr">
         <is>
-          <t>831069081846626</t>
+          <t>502048965091595</t>
         </is>
       </c>
       <c r="AL2" s="32" t="inlineStr">

</xml_diff>

<commit_message>
fix: restore scripts and fix import errors (clean)
</commit_message>
<xml_diff>
--- a/Data/LOSData.xlsx
+++ b/Data/LOSData.xlsx
@@ -1001,7 +1001,7 @@
     <row r="2" ht="19.5" customHeight="1" thickBot="1">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>0001911094169</t>
+          <t>0001911094337</t>
         </is>
       </c>
       <c r="B2" s="37" t="inlineStr">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H2" s="20" t="inlineStr">
         <is>
-          <t>Brianna Joe</t>
+          <t>DANIEL</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Brianna</t>
+          <t>DANIEL</t>
         </is>
       </c>
       <c r="J2" s="22" t="n">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="P2" s="28" t="inlineStr">
         <is>
-          <t>4428444224168525</t>
+          <t>6212299659498981</t>
         </is>
       </c>
       <c r="Q2" s="25" t="n">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="T2" s="20" t="inlineStr">
         <is>
-          <t>Levi Ward</t>
+          <t>Anne Ward</t>
         </is>
       </c>
       <c r="U2" s="25" t="n">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="AK2" s="28" t="inlineStr">
         <is>
-          <t>502048965091595</t>
+          <t>387072122621185</t>
         </is>
       </c>
       <c r="AL2" s="32" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="AM2" s="23" t="inlineStr">
         <is>
-          <t>KNP2026022000029</t>
+          <t>KNP2026032500001</t>
         </is>
       </c>
     </row>

</xml_diff>